<commit_message>
Actualizacion datos REM 2026-09-29 16:23 (orquestador)
</commit_message>
<xml_diff>
--- a/output/2017-2026_A03_SECCION_A5_TABLAS.xlsx
+++ b/output/2017-2026_A03_SECCION_A5_TABLAS.xlsx
@@ -729,16 +729,16 @@
         <v>14</v>
       </c>
       <c r="B11">
-        <v>13440</v>
+        <v>21496</v>
       </c>
       <c r="C11">
-        <v>8294</v>
+        <v>13252</v>
       </c>
       <c r="D11" t="s">
         <v>15</v>
       </c>
       <c r="E11">
-        <v>61.71</v>
+        <v>61.65</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -8563,16 +8563,16 @@
         <v>14</v>
       </c>
       <c r="B472">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C472">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D472" t="s">
         <v>16</v>
       </c>
       <c r="E472">
-        <v>50</v>
+        <v>47.37</v>
       </c>
     </row>
     <row r="473" spans="1:5">
@@ -8580,16 +8580,16 @@
         <v>14</v>
       </c>
       <c r="B473">
-        <v>157</v>
+        <v>258</v>
       </c>
       <c r="C473">
-        <v>112</v>
+        <v>180</v>
       </c>
       <c r="D473" t="s">
         <v>17</v>
       </c>
       <c r="E473">
-        <v>71.34</v>
+        <v>69.77</v>
       </c>
     </row>
     <row r="474" spans="1:5">
@@ -8597,16 +8597,16 @@
         <v>14</v>
       </c>
       <c r="B474">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="C474">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="D474" t="s">
         <v>18</v>
       </c>
       <c r="E474">
-        <v>62.5</v>
+        <v>64.29000000000001</v>
       </c>
     </row>
     <row r="475" spans="1:5">
@@ -8614,16 +8614,16 @@
         <v>14</v>
       </c>
       <c r="B475">
-        <v>168</v>
+        <v>290</v>
       </c>
       <c r="C475">
-        <v>124</v>
+        <v>213</v>
       </c>
       <c r="D475" t="s">
         <v>19</v>
       </c>
       <c r="E475">
-        <v>73.81</v>
+        <v>73.45</v>
       </c>
     </row>
     <row r="476" spans="1:5">
@@ -8631,16 +8631,16 @@
         <v>14</v>
       </c>
       <c r="B476">
-        <v>324</v>
+        <v>516</v>
       </c>
       <c r="C476">
-        <v>209</v>
+        <v>330</v>
       </c>
       <c r="D476" t="s">
         <v>20</v>
       </c>
       <c r="E476">
-        <v>64.51000000000001</v>
+        <v>63.95</v>
       </c>
     </row>
     <row r="477" spans="1:5">
@@ -8648,16 +8648,16 @@
         <v>14</v>
       </c>
       <c r="B477">
-        <v>386</v>
+        <v>630</v>
       </c>
       <c r="C477">
-        <v>222</v>
+        <v>387</v>
       </c>
       <c r="D477" t="s">
         <v>21</v>
       </c>
       <c r="E477">
-        <v>57.51</v>
+        <v>61.43</v>
       </c>
     </row>
     <row r="478" spans="1:5">
@@ -8665,16 +8665,16 @@
         <v>14</v>
       </c>
       <c r="B478">
-        <v>273</v>
+        <v>438</v>
       </c>
       <c r="C478">
-        <v>164</v>
+        <v>263</v>
       </c>
       <c r="D478" t="s">
         <v>22</v>
       </c>
       <c r="E478">
-        <v>60.07</v>
+        <v>60.05</v>
       </c>
     </row>
     <row r="479" spans="1:5">
@@ -8682,16 +8682,16 @@
         <v>14</v>
       </c>
       <c r="B479">
-        <v>89</v>
+        <v>142</v>
       </c>
       <c r="C479">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="D479" t="s">
         <v>23</v>
       </c>
       <c r="E479">
-        <v>55.06</v>
+        <v>60.56</v>
       </c>
     </row>
     <row r="480" spans="1:5">
@@ -8699,16 +8699,16 @@
         <v>14</v>
       </c>
       <c r="B480">
-        <v>374</v>
+        <v>587</v>
       </c>
       <c r="C480">
-        <v>219</v>
+        <v>341</v>
       </c>
       <c r="D480" t="s">
         <v>24</v>
       </c>
       <c r="E480">
-        <v>58.56</v>
+        <v>58.09</v>
       </c>
     </row>
     <row r="481" spans="1:5">
@@ -8716,16 +8716,16 @@
         <v>14</v>
       </c>
       <c r="B481">
-        <v>92</v>
+        <v>131</v>
       </c>
       <c r="C481">
-        <v>63</v>
+        <v>86</v>
       </c>
       <c r="D481" t="s">
         <v>25</v>
       </c>
       <c r="E481">
-        <v>68.48</v>
+        <v>65.65000000000001</v>
       </c>
     </row>
     <row r="482" spans="1:5">
@@ -8733,16 +8733,16 @@
         <v>14</v>
       </c>
       <c r="B482">
-        <v>395</v>
+        <v>638</v>
       </c>
       <c r="C482">
-        <v>276</v>
+        <v>462</v>
       </c>
       <c r="D482" t="s">
         <v>26</v>
       </c>
       <c r="E482">
-        <v>69.87</v>
+        <v>72.41</v>
       </c>
     </row>
     <row r="483" spans="1:5">
@@ -8750,16 +8750,16 @@
         <v>14</v>
       </c>
       <c r="B483">
-        <v>196</v>
+        <v>303</v>
       </c>
       <c r="C483">
-        <v>134</v>
+        <v>206</v>
       </c>
       <c r="D483" t="s">
         <v>27</v>
       </c>
       <c r="E483">
-        <v>68.37</v>
+        <v>67.98999999999999</v>
       </c>
     </row>
     <row r="484" spans="1:5">
@@ -8767,16 +8767,16 @@
         <v>14</v>
       </c>
       <c r="B484">
-        <v>360</v>
+        <v>590</v>
       </c>
       <c r="C484">
-        <v>247</v>
+        <v>402</v>
       </c>
       <c r="D484" t="s">
         <v>28</v>
       </c>
       <c r="E484">
-        <v>68.61</v>
+        <v>68.14</v>
       </c>
     </row>
     <row r="485" spans="1:5">
@@ -8784,16 +8784,16 @@
         <v>14</v>
       </c>
       <c r="B485">
-        <v>100</v>
+        <v>183</v>
       </c>
       <c r="C485">
-        <v>56</v>
+        <v>103</v>
       </c>
       <c r="D485" t="s">
         <v>29</v>
       </c>
       <c r="E485">
-        <v>56</v>
+        <v>56.28</v>
       </c>
     </row>
     <row r="486" spans="1:5">
@@ -8801,16 +8801,16 @@
         <v>14</v>
       </c>
       <c r="B486">
-        <v>223</v>
+        <v>334</v>
       </c>
       <c r="C486">
-        <v>133</v>
+        <v>190</v>
       </c>
       <c r="D486" t="s">
         <v>30</v>
       </c>
       <c r="E486">
-        <v>59.64</v>
+        <v>56.89</v>
       </c>
     </row>
     <row r="487" spans="1:5">
@@ -8818,16 +8818,16 @@
         <v>14</v>
       </c>
       <c r="B487">
-        <v>928</v>
+        <v>1429</v>
       </c>
       <c r="C487">
-        <v>546</v>
+        <v>836</v>
       </c>
       <c r="D487" t="s">
         <v>31</v>
       </c>
       <c r="E487">
-        <v>58.84</v>
+        <v>58.5</v>
       </c>
     </row>
     <row r="488" spans="1:5">
@@ -8835,16 +8835,16 @@
         <v>14</v>
       </c>
       <c r="B488">
-        <v>245</v>
+        <v>396</v>
       </c>
       <c r="C488">
-        <v>157</v>
+        <v>242</v>
       </c>
       <c r="D488" t="s">
         <v>32</v>
       </c>
       <c r="E488">
-        <v>64.08</v>
+        <v>61.11</v>
       </c>
     </row>
     <row r="489" spans="1:5">
@@ -8852,16 +8852,16 @@
         <v>14</v>
       </c>
       <c r="B489">
-        <v>383</v>
+        <v>617</v>
       </c>
       <c r="C489">
-        <v>214</v>
+        <v>363</v>
       </c>
       <c r="D489" t="s">
         <v>33</v>
       </c>
       <c r="E489">
-        <v>55.87</v>
+        <v>58.83</v>
       </c>
     </row>
     <row r="490" spans="1:5">
@@ -8869,16 +8869,16 @@
         <v>14</v>
       </c>
       <c r="B490">
-        <v>78</v>
+        <v>124</v>
       </c>
       <c r="C490">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="D490" t="s">
         <v>34</v>
       </c>
       <c r="E490">
-        <v>58.97</v>
+        <v>59.68</v>
       </c>
     </row>
     <row r="491" spans="1:5">
@@ -8886,16 +8886,16 @@
         <v>14</v>
       </c>
       <c r="B491">
-        <v>315</v>
+        <v>489</v>
       </c>
       <c r="C491">
-        <v>193</v>
+        <v>289</v>
       </c>
       <c r="D491" t="s">
         <v>35</v>
       </c>
       <c r="E491">
-        <v>61.27</v>
+        <v>59.1</v>
       </c>
     </row>
     <row r="492" spans="1:5">
@@ -8903,16 +8903,16 @@
         <v>14</v>
       </c>
       <c r="B492">
-        <v>91</v>
+        <v>148</v>
       </c>
       <c r="C492">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="D492" t="s">
         <v>36</v>
       </c>
       <c r="E492">
-        <v>43.96</v>
+        <v>52.03</v>
       </c>
     </row>
     <row r="493" spans="1:5">
@@ -8920,16 +8920,16 @@
         <v>14</v>
       </c>
       <c r="B493">
-        <v>87</v>
+        <v>151</v>
       </c>
       <c r="C493">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="D493" t="s">
         <v>37</v>
       </c>
       <c r="E493">
-        <v>45.98</v>
+        <v>51.66</v>
       </c>
     </row>
     <row r="494" spans="1:5">
@@ -8937,16 +8937,16 @@
         <v>14</v>
       </c>
       <c r="B494">
-        <v>234</v>
+        <v>369</v>
       </c>
       <c r="C494">
-        <v>143</v>
+        <v>231</v>
       </c>
       <c r="D494" t="s">
         <v>38</v>
       </c>
       <c r="E494">
-        <v>61.11</v>
+        <v>62.6</v>
       </c>
     </row>
     <row r="495" spans="1:5">
@@ -8954,16 +8954,16 @@
         <v>14</v>
       </c>
       <c r="B495">
-        <v>275</v>
+        <v>420</v>
       </c>
       <c r="C495">
-        <v>155</v>
+        <v>229</v>
       </c>
       <c r="D495" t="s">
         <v>39</v>
       </c>
       <c r="E495">
-        <v>56.36</v>
+        <v>54.52</v>
       </c>
     </row>
     <row r="496" spans="1:5">
@@ -8971,16 +8971,16 @@
         <v>14</v>
       </c>
       <c r="B496">
-        <v>187</v>
+        <v>289</v>
       </c>
       <c r="C496">
-        <v>127</v>
+        <v>198</v>
       </c>
       <c r="D496" t="s">
         <v>40</v>
       </c>
       <c r="E496">
-        <v>67.91</v>
+        <v>68.51000000000001</v>
       </c>
     </row>
     <row r="497" spans="1:5">
@@ -8988,16 +8988,16 @@
         <v>14</v>
       </c>
       <c r="B497">
-        <v>746</v>
+        <v>1168</v>
       </c>
       <c r="C497">
-        <v>442</v>
+        <v>677</v>
       </c>
       <c r="D497" t="s">
         <v>41</v>
       </c>
       <c r="E497">
-        <v>59.25</v>
+        <v>57.96</v>
       </c>
     </row>
     <row r="498" spans="1:5">
@@ -9005,16 +9005,16 @@
         <v>14</v>
       </c>
       <c r="B498">
-        <v>48</v>
+        <v>77</v>
       </c>
       <c r="C498">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="D498" t="s">
         <v>42</v>
       </c>
       <c r="E498">
-        <v>54.17</v>
+        <v>49.35</v>
       </c>
     </row>
     <row r="499" spans="1:5">
@@ -9022,16 +9022,16 @@
         <v>14</v>
       </c>
       <c r="B499">
-        <v>293</v>
+        <v>460</v>
       </c>
       <c r="C499">
-        <v>185</v>
+        <v>309</v>
       </c>
       <c r="D499" t="s">
         <v>43</v>
       </c>
       <c r="E499">
-        <v>63.14</v>
+        <v>67.17</v>
       </c>
     </row>
     <row r="500" spans="1:5">
@@ -9039,16 +9039,16 @@
         <v>14</v>
       </c>
       <c r="B500">
-        <v>129</v>
+        <v>201</v>
       </c>
       <c r="C500">
-        <v>80</v>
+        <v>122</v>
       </c>
       <c r="D500" t="s">
         <v>44</v>
       </c>
       <c r="E500">
-        <v>62.02</v>
+        <v>60.7</v>
       </c>
     </row>
     <row r="501" spans="1:5">
@@ -9056,16 +9056,16 @@
         <v>14</v>
       </c>
       <c r="B501">
-        <v>205</v>
+        <v>304</v>
       </c>
       <c r="C501">
-        <v>134</v>
+        <v>202</v>
       </c>
       <c r="D501" t="s">
         <v>45</v>
       </c>
       <c r="E501">
-        <v>65.37</v>
+        <v>66.45</v>
       </c>
     </row>
     <row r="502" spans="1:5">
@@ -9073,16 +9073,16 @@
         <v>14</v>
       </c>
       <c r="B502">
-        <v>216</v>
+        <v>340</v>
       </c>
       <c r="C502">
-        <v>136</v>
+        <v>210</v>
       </c>
       <c r="D502" t="s">
         <v>46</v>
       </c>
       <c r="E502">
-        <v>62.96</v>
+        <v>61.76</v>
       </c>
     </row>
     <row r="503" spans="1:5">
@@ -9090,16 +9090,16 @@
         <v>14</v>
       </c>
       <c r="B503">
-        <v>177</v>
+        <v>294</v>
       </c>
       <c r="C503">
-        <v>129</v>
+        <v>211</v>
       </c>
       <c r="D503" t="s">
         <v>47</v>
       </c>
       <c r="E503">
-        <v>72.88</v>
+        <v>71.77</v>
       </c>
     </row>
     <row r="504" spans="1:5">
@@ -9107,16 +9107,16 @@
         <v>14</v>
       </c>
       <c r="B504">
-        <v>437</v>
+        <v>699</v>
       </c>
       <c r="C504">
-        <v>269</v>
+        <v>433</v>
       </c>
       <c r="D504" t="s">
         <v>48</v>
       </c>
       <c r="E504">
-        <v>61.56</v>
+        <v>61.95</v>
       </c>
     </row>
     <row r="505" spans="1:5">
@@ -9124,16 +9124,16 @@
         <v>14</v>
       </c>
       <c r="B505">
-        <v>47</v>
+        <v>84</v>
       </c>
       <c r="C505">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="D505" t="s">
         <v>49</v>
       </c>
       <c r="E505">
-        <v>48.94</v>
+        <v>54.76</v>
       </c>
     </row>
     <row r="506" spans="1:5">
@@ -9141,16 +9141,16 @@
         <v>14</v>
       </c>
       <c r="B506">
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="C506">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="D506" t="s">
         <v>50</v>
       </c>
       <c r="E506">
-        <v>61.54</v>
+        <v>64</v>
       </c>
     </row>
     <row r="507" spans="1:5">
@@ -9158,16 +9158,16 @@
         <v>14</v>
       </c>
       <c r="B507">
-        <v>375</v>
+        <v>608</v>
       </c>
       <c r="C507">
-        <v>223</v>
+        <v>358</v>
       </c>
       <c r="D507" t="s">
         <v>51</v>
       </c>
       <c r="E507">
-        <v>59.47</v>
+        <v>58.88</v>
       </c>
     </row>
     <row r="508" spans="1:5">
@@ -9175,16 +9175,16 @@
         <v>14</v>
       </c>
       <c r="B508">
-        <v>782</v>
+        <v>1301</v>
       </c>
       <c r="C508">
-        <v>445</v>
+        <v>707</v>
       </c>
       <c r="D508" t="s">
         <v>52</v>
       </c>
       <c r="E508">
-        <v>56.91</v>
+        <v>54.34</v>
       </c>
     </row>
     <row r="509" spans="1:5">
@@ -9192,16 +9192,16 @@
         <v>14</v>
       </c>
       <c r="B509">
-        <v>500</v>
+        <v>814</v>
       </c>
       <c r="C509">
-        <v>314</v>
+        <v>517</v>
       </c>
       <c r="D509" t="s">
         <v>53</v>
       </c>
       <c r="E509">
-        <v>62.8</v>
+        <v>63.51</v>
       </c>
     </row>
     <row r="510" spans="1:5">
@@ -9209,16 +9209,16 @@
         <v>14</v>
       </c>
       <c r="B510">
-        <v>262</v>
+        <v>391</v>
       </c>
       <c r="C510">
-        <v>159</v>
+        <v>246</v>
       </c>
       <c r="D510" t="s">
         <v>54</v>
       </c>
       <c r="E510">
-        <v>60.69</v>
+        <v>62.92</v>
       </c>
     </row>
     <row r="511" spans="1:5">
@@ -9226,16 +9226,16 @@
         <v>14</v>
       </c>
       <c r="B511">
-        <v>331</v>
+        <v>521</v>
       </c>
       <c r="C511">
-        <v>210</v>
+        <v>321</v>
       </c>
       <c r="D511" t="s">
         <v>55</v>
       </c>
       <c r="E511">
-        <v>63.44</v>
+        <v>61.61</v>
       </c>
     </row>
     <row r="512" spans="1:5">
@@ -9243,16 +9243,16 @@
         <v>14</v>
       </c>
       <c r="B512">
-        <v>357</v>
+        <v>621</v>
       </c>
       <c r="C512">
-        <v>228</v>
+        <v>399</v>
       </c>
       <c r="D512" t="s">
         <v>56</v>
       </c>
       <c r="E512">
-        <v>63.87</v>
+        <v>64.25</v>
       </c>
     </row>
     <row r="513" spans="1:5">
@@ -9260,16 +9260,16 @@
         <v>14</v>
       </c>
       <c r="B513">
-        <v>577</v>
+        <v>904</v>
       </c>
       <c r="C513">
-        <v>336</v>
+        <v>516</v>
       </c>
       <c r="D513" t="s">
         <v>57</v>
       </c>
       <c r="E513">
-        <v>58.23</v>
+        <v>57.08</v>
       </c>
     </row>
     <row r="514" spans="1:5">
@@ -9277,16 +9277,16 @@
         <v>14</v>
       </c>
       <c r="B514">
-        <v>165</v>
+        <v>254</v>
       </c>
       <c r="C514">
-        <v>96</v>
+        <v>146</v>
       </c>
       <c r="D514" t="s">
         <v>58</v>
       </c>
       <c r="E514">
-        <v>58.18</v>
+        <v>57.48</v>
       </c>
     </row>
     <row r="515" spans="1:5">
@@ -9294,16 +9294,16 @@
         <v>14</v>
       </c>
       <c r="B515">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="C515">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D515" t="s">
         <v>59</v>
       </c>
       <c r="E515">
-        <v>59.46</v>
+        <v>64.81</v>
       </c>
     </row>
     <row r="516" spans="1:5">
@@ -9311,16 +9311,16 @@
         <v>14</v>
       </c>
       <c r="B516">
-        <v>231</v>
+        <v>401</v>
       </c>
       <c r="C516">
-        <v>141</v>
+        <v>239</v>
       </c>
       <c r="D516" t="s">
         <v>60</v>
       </c>
       <c r="E516">
-        <v>61.04</v>
+        <v>59.6</v>
       </c>
     </row>
     <row r="517" spans="1:5">
@@ -9328,16 +9328,16 @@
         <v>14</v>
       </c>
       <c r="B517">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="C517">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="D517" t="s">
         <v>61</v>
       </c>
       <c r="E517">
-        <v>60.87</v>
+        <v>69.23</v>
       </c>
     </row>
     <row r="518" spans="1:5">
@@ -9345,16 +9345,16 @@
         <v>14</v>
       </c>
       <c r="B518">
-        <v>190</v>
+        <v>288</v>
       </c>
       <c r="C518">
-        <v>146</v>
+        <v>221</v>
       </c>
       <c r="D518" t="s">
         <v>62</v>
       </c>
       <c r="E518">
-        <v>76.84</v>
+        <v>76.73999999999999</v>
       </c>
     </row>
     <row r="519" spans="1:5">
@@ -9362,16 +9362,16 @@
         <v>14</v>
       </c>
       <c r="B519">
-        <v>860</v>
+        <v>1416</v>
       </c>
       <c r="C519">
-        <v>541</v>
+        <v>901</v>
       </c>
       <c r="D519" t="s">
         <v>63</v>
       </c>
       <c r="E519">
-        <v>62.91</v>
+        <v>63.63</v>
       </c>
     </row>
     <row r="520" spans="1:5">
@@ -9379,16 +9379,16 @@
         <v>14</v>
       </c>
       <c r="B520">
-        <v>118</v>
+        <v>202</v>
       </c>
       <c r="C520">
-        <v>76</v>
+        <v>123</v>
       </c>
       <c r="D520" t="s">
         <v>64</v>
       </c>
       <c r="E520">
-        <v>64.41</v>
+        <v>60.89</v>
       </c>
     </row>
     <row r="521" spans="1:5">
@@ -9396,16 +9396,16 @@
         <v>14</v>
       </c>
       <c r="B521">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="C521">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="D521" t="s">
         <v>65</v>
       </c>
       <c r="E521">
-        <v>90.7</v>
+        <v>80.28</v>
       </c>
     </row>
     <row r="522" spans="1:5">
@@ -9413,16 +9413,16 @@
         <v>14</v>
       </c>
       <c r="B522">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="C522">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D522" t="s">
         <v>66</v>
       </c>
       <c r="E522">
-        <v>50</v>
+        <v>40.74</v>
       </c>
     </row>
     <row r="523" spans="1:5">
@@ -9430,16 +9430,16 @@
         <v>14</v>
       </c>
       <c r="B523">
-        <v>198</v>
+        <v>310</v>
       </c>
       <c r="C523">
-        <v>132</v>
+        <v>205</v>
       </c>
       <c r="D523" t="s">
         <v>67</v>
       </c>
       <c r="E523">
-        <v>66.67</v>
+        <v>66.13</v>
       </c>
     </row>
   </sheetData>
@@ -9627,16 +9627,16 @@
         <v>14</v>
       </c>
       <c r="B11">
-        <v>12578</v>
+        <v>20702</v>
       </c>
       <c r="C11">
-        <v>7205</v>
+        <v>11754</v>
       </c>
       <c r="D11" t="s">
         <v>15</v>
       </c>
       <c r="E11">
-        <v>57.28</v>
+        <v>56.78</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -17461,16 +17461,16 @@
         <v>14</v>
       </c>
       <c r="B472">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C472">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D472" t="s">
         <v>16</v>
       </c>
       <c r="E472">
-        <v>44.44</v>
+        <v>58.82</v>
       </c>
     </row>
     <row r="473" spans="1:5">
@@ -17478,16 +17478,16 @@
         <v>14</v>
       </c>
       <c r="B473">
-        <v>173</v>
+        <v>274</v>
       </c>
       <c r="C473">
-        <v>95</v>
+        <v>152</v>
       </c>
       <c r="D473" t="s">
         <v>17</v>
       </c>
       <c r="E473">
-        <v>54.91</v>
+        <v>55.47</v>
       </c>
     </row>
     <row r="474" spans="1:5">
@@ -17495,16 +17495,16 @@
         <v>14</v>
       </c>
       <c r="B474">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="C474">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="D474" t="s">
         <v>18</v>
       </c>
       <c r="E474">
-        <v>56.1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="475" spans="1:5">
@@ -17512,16 +17512,16 @@
         <v>14</v>
       </c>
       <c r="B475">
-        <v>146</v>
+        <v>240</v>
       </c>
       <c r="C475">
-        <v>96</v>
+        <v>157</v>
       </c>
       <c r="D475" t="s">
         <v>19</v>
       </c>
       <c r="E475">
-        <v>65.75</v>
+        <v>65.42</v>
       </c>
     </row>
     <row r="476" spans="1:5">
@@ -17529,16 +17529,16 @@
         <v>14</v>
       </c>
       <c r="B476">
-        <v>294</v>
+        <v>500</v>
       </c>
       <c r="C476">
-        <v>161</v>
+        <v>277</v>
       </c>
       <c r="D476" t="s">
         <v>20</v>
       </c>
       <c r="E476">
-        <v>54.76</v>
+        <v>55.4</v>
       </c>
     </row>
     <row r="477" spans="1:5">
@@ -17546,16 +17546,16 @@
         <v>14</v>
       </c>
       <c r="B477">
-        <v>330</v>
+        <v>557</v>
       </c>
       <c r="C477">
-        <v>187</v>
+        <v>322</v>
       </c>
       <c r="D477" t="s">
         <v>21</v>
       </c>
       <c r="E477">
-        <v>56.67</v>
+        <v>57.81</v>
       </c>
     </row>
     <row r="478" spans="1:5">
@@ -17563,16 +17563,16 @@
         <v>14</v>
       </c>
       <c r="B478">
-        <v>262</v>
+        <v>430</v>
       </c>
       <c r="C478">
-        <v>145</v>
+        <v>231</v>
       </c>
       <c r="D478" t="s">
         <v>22</v>
       </c>
       <c r="E478">
-        <v>55.34</v>
+        <v>53.72</v>
       </c>
     </row>
     <row r="479" spans="1:5">
@@ -17580,16 +17580,16 @@
         <v>14</v>
       </c>
       <c r="B479">
-        <v>85</v>
+        <v>132</v>
       </c>
       <c r="C479">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="D479" t="s">
         <v>23</v>
       </c>
       <c r="E479">
-        <v>55.29</v>
+        <v>59.09</v>
       </c>
     </row>
     <row r="480" spans="1:5">
@@ -17597,16 +17597,16 @@
         <v>14</v>
       </c>
       <c r="B480">
-        <v>345</v>
+        <v>587</v>
       </c>
       <c r="C480">
-        <v>168</v>
+        <v>296</v>
       </c>
       <c r="D480" t="s">
         <v>24</v>
       </c>
       <c r="E480">
-        <v>48.7</v>
+        <v>50.43</v>
       </c>
     </row>
     <row r="481" spans="1:5">
@@ -17614,16 +17614,16 @@
         <v>14</v>
       </c>
       <c r="B481">
-        <v>73</v>
+        <v>117</v>
       </c>
       <c r="C481">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="D481" t="s">
         <v>25</v>
       </c>
       <c r="E481">
-        <v>60.27</v>
+        <v>65.81</v>
       </c>
     </row>
     <row r="482" spans="1:5">
@@ -17631,16 +17631,16 @@
         <v>14</v>
       </c>
       <c r="B482">
-        <v>338</v>
+        <v>584</v>
       </c>
       <c r="C482">
-        <v>213</v>
+        <v>369</v>
       </c>
       <c r="D482" t="s">
         <v>26</v>
       </c>
       <c r="E482">
-        <v>63.02</v>
+        <v>63.18</v>
       </c>
     </row>
     <row r="483" spans="1:5">
@@ -17648,16 +17648,16 @@
         <v>14</v>
       </c>
       <c r="B483">
-        <v>181</v>
+        <v>305</v>
       </c>
       <c r="C483">
-        <v>115</v>
+        <v>190</v>
       </c>
       <c r="D483" t="s">
         <v>27</v>
       </c>
       <c r="E483">
-        <v>63.54</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="484" spans="1:5">
@@ -17665,16 +17665,16 @@
         <v>14</v>
       </c>
       <c r="B484">
-        <v>361</v>
+        <v>593</v>
       </c>
       <c r="C484">
-        <v>245</v>
+        <v>391</v>
       </c>
       <c r="D484" t="s">
         <v>28</v>
       </c>
       <c r="E484">
-        <v>67.87</v>
+        <v>65.94</v>
       </c>
     </row>
     <row r="485" spans="1:5">
@@ -17682,16 +17682,16 @@
         <v>14</v>
       </c>
       <c r="B485">
-        <v>84</v>
+        <v>164</v>
       </c>
       <c r="C485">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="D485" t="s">
         <v>29</v>
       </c>
       <c r="E485">
-        <v>61.9</v>
+        <v>53.66</v>
       </c>
     </row>
     <row r="486" spans="1:5">
@@ -17699,16 +17699,16 @@
         <v>14</v>
       </c>
       <c r="B486">
-        <v>209</v>
+        <v>327</v>
       </c>
       <c r="C486">
-        <v>113</v>
+        <v>172</v>
       </c>
       <c r="D486" t="s">
         <v>30</v>
       </c>
       <c r="E486">
-        <v>54.07</v>
+        <v>52.6</v>
       </c>
     </row>
     <row r="487" spans="1:5">
@@ -17716,16 +17716,16 @@
         <v>14</v>
       </c>
       <c r="B487">
-        <v>853</v>
+        <v>1383</v>
       </c>
       <c r="C487">
-        <v>512</v>
+        <v>781</v>
       </c>
       <c r="D487" t="s">
         <v>31</v>
       </c>
       <c r="E487">
-        <v>60.02</v>
+        <v>56.47</v>
       </c>
     </row>
     <row r="488" spans="1:5">
@@ -17733,16 +17733,16 @@
         <v>14</v>
       </c>
       <c r="B488">
-        <v>228</v>
+        <v>373</v>
       </c>
       <c r="C488">
-        <v>103</v>
+        <v>176</v>
       </c>
       <c r="D488" t="s">
         <v>32</v>
       </c>
       <c r="E488">
-        <v>45.18</v>
+        <v>47.18</v>
       </c>
     </row>
     <row r="489" spans="1:5">
@@ -17750,16 +17750,16 @@
         <v>14</v>
       </c>
       <c r="B489">
-        <v>342</v>
+        <v>561</v>
       </c>
       <c r="C489">
-        <v>167</v>
+        <v>285</v>
       </c>
       <c r="D489" t="s">
         <v>33</v>
       </c>
       <c r="E489">
-        <v>48.83</v>
+        <v>50.8</v>
       </c>
     </row>
     <row r="490" spans="1:5">
@@ -17767,16 +17767,16 @@
         <v>14</v>
       </c>
       <c r="B490">
-        <v>73</v>
+        <v>118</v>
       </c>
       <c r="C490">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="D490" t="s">
         <v>34</v>
       </c>
       <c r="E490">
-        <v>43.84</v>
+        <v>45.76</v>
       </c>
     </row>
     <row r="491" spans="1:5">
@@ -17784,16 +17784,16 @@
         <v>14</v>
       </c>
       <c r="B491">
-        <v>298</v>
+        <v>510</v>
       </c>
       <c r="C491">
-        <v>158</v>
+        <v>289</v>
       </c>
       <c r="D491" t="s">
         <v>35</v>
       </c>
       <c r="E491">
-        <v>53.02</v>
+        <v>56.67</v>
       </c>
     </row>
     <row r="492" spans="1:5">
@@ -17801,16 +17801,16 @@
         <v>14</v>
       </c>
       <c r="B492">
-        <v>93</v>
+        <v>150</v>
       </c>
       <c r="C492">
-        <v>44</v>
+        <v>73</v>
       </c>
       <c r="D492" t="s">
         <v>36</v>
       </c>
       <c r="E492">
-        <v>47.31</v>
+        <v>48.67</v>
       </c>
     </row>
     <row r="493" spans="1:5">
@@ -17818,16 +17818,16 @@
         <v>14</v>
       </c>
       <c r="B493">
-        <v>96</v>
+        <v>149</v>
       </c>
       <c r="C493">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="D493" t="s">
         <v>37</v>
       </c>
       <c r="E493">
-        <v>44.79</v>
+        <v>47.65</v>
       </c>
     </row>
     <row r="494" spans="1:5">
@@ -17835,16 +17835,16 @@
         <v>14</v>
       </c>
       <c r="B494">
-        <v>166</v>
+        <v>272</v>
       </c>
       <c r="C494">
-        <v>99</v>
+        <v>162</v>
       </c>
       <c r="D494" t="s">
         <v>38</v>
       </c>
       <c r="E494">
-        <v>59.64</v>
+        <v>59.56</v>
       </c>
     </row>
     <row r="495" spans="1:5">
@@ -17852,16 +17852,16 @@
         <v>14</v>
       </c>
       <c r="B495">
-        <v>220</v>
+        <v>402</v>
       </c>
       <c r="C495">
-        <v>136</v>
+        <v>227</v>
       </c>
       <c r="D495" t="s">
         <v>39</v>
       </c>
       <c r="E495">
-        <v>61.82</v>
+        <v>56.47</v>
       </c>
     </row>
     <row r="496" spans="1:5">
@@ -17869,16 +17869,16 @@
         <v>14</v>
       </c>
       <c r="B496">
-        <v>171</v>
+        <v>273</v>
       </c>
       <c r="C496">
-        <v>97</v>
+        <v>174</v>
       </c>
       <c r="D496" t="s">
         <v>40</v>
       </c>
       <c r="E496">
-        <v>56.73</v>
+        <v>63.74</v>
       </c>
     </row>
     <row r="497" spans="1:5">
@@ -17886,16 +17886,16 @@
         <v>14</v>
       </c>
       <c r="B497">
-        <v>607</v>
+        <v>978</v>
       </c>
       <c r="C497">
-        <v>328</v>
+        <v>512</v>
       </c>
       <c r="D497" t="s">
         <v>41</v>
       </c>
       <c r="E497">
-        <v>54.04</v>
+        <v>52.35</v>
       </c>
     </row>
     <row r="498" spans="1:5">
@@ -17903,16 +17903,16 @@
         <v>14</v>
       </c>
       <c r="B498">
-        <v>48</v>
+        <v>73</v>
       </c>
       <c r="C498">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="D498" t="s">
         <v>42</v>
       </c>
       <c r="E498">
-        <v>56.25</v>
+        <v>54.79</v>
       </c>
     </row>
     <row r="499" spans="1:5">
@@ -17920,16 +17920,16 @@
         <v>14</v>
       </c>
       <c r="B499">
-        <v>282</v>
+        <v>438</v>
       </c>
       <c r="C499">
-        <v>164</v>
+        <v>271</v>
       </c>
       <c r="D499" t="s">
         <v>43</v>
       </c>
       <c r="E499">
-        <v>58.16</v>
+        <v>61.87</v>
       </c>
     </row>
     <row r="500" spans="1:5">
@@ -17937,16 +17937,16 @@
         <v>14</v>
       </c>
       <c r="B500">
-        <v>115</v>
+        <v>207</v>
       </c>
       <c r="C500">
-        <v>75</v>
+        <v>126</v>
       </c>
       <c r="D500" t="s">
         <v>44</v>
       </c>
       <c r="E500">
-        <v>65.22</v>
+        <v>60.87</v>
       </c>
     </row>
     <row r="501" spans="1:5">
@@ -17954,16 +17954,16 @@
         <v>14</v>
       </c>
       <c r="B501">
-        <v>225</v>
+        <v>321</v>
       </c>
       <c r="C501">
-        <v>132</v>
+        <v>194</v>
       </c>
       <c r="D501" t="s">
         <v>45</v>
       </c>
       <c r="E501">
-        <v>58.67</v>
+        <v>60.44</v>
       </c>
     </row>
     <row r="502" spans="1:5">
@@ -17971,16 +17971,16 @@
         <v>14</v>
       </c>
       <c r="B502">
-        <v>197</v>
+        <v>336</v>
       </c>
       <c r="C502">
-        <v>120</v>
+        <v>194</v>
       </c>
       <c r="D502" t="s">
         <v>46</v>
       </c>
       <c r="E502">
-        <v>60.91</v>
+        <v>57.74</v>
       </c>
     </row>
     <row r="503" spans="1:5">
@@ -17988,16 +17988,16 @@
         <v>14</v>
       </c>
       <c r="B503">
-        <v>143</v>
+        <v>243</v>
       </c>
       <c r="C503">
-        <v>97</v>
+        <v>160</v>
       </c>
       <c r="D503" t="s">
         <v>47</v>
       </c>
       <c r="E503">
-        <v>67.83</v>
+        <v>65.84</v>
       </c>
     </row>
     <row r="504" spans="1:5">
@@ -18005,16 +18005,16 @@
         <v>14</v>
       </c>
       <c r="B504">
-        <v>363</v>
+        <v>615</v>
       </c>
       <c r="C504">
-        <v>225</v>
+        <v>361</v>
       </c>
       <c r="D504" t="s">
         <v>48</v>
       </c>
       <c r="E504">
-        <v>61.98</v>
+        <v>58.7</v>
       </c>
     </row>
     <row r="505" spans="1:5">
@@ -18022,16 +18022,16 @@
         <v>14</v>
       </c>
       <c r="B505">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="C505">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="D505" t="s">
         <v>49</v>
       </c>
       <c r="E505">
-        <v>54.55</v>
+        <v>55.22</v>
       </c>
     </row>
     <row r="506" spans="1:5">
@@ -18039,16 +18039,16 @@
         <v>14</v>
       </c>
       <c r="B506">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="C506">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D506" t="s">
         <v>50</v>
       </c>
       <c r="E506">
-        <v>70.37</v>
+        <v>70.93000000000001</v>
       </c>
     </row>
     <row r="507" spans="1:5">
@@ -18056,16 +18056,16 @@
         <v>14</v>
       </c>
       <c r="B507">
-        <v>409</v>
+        <v>720</v>
       </c>
       <c r="C507">
-        <v>241</v>
+        <v>432</v>
       </c>
       <c r="D507" t="s">
         <v>51</v>
       </c>
       <c r="E507">
-        <v>58.92</v>
+        <v>60</v>
       </c>
     </row>
     <row r="508" spans="1:5">
@@ -18073,16 +18073,16 @@
         <v>14</v>
       </c>
       <c r="B508">
-        <v>737</v>
+        <v>1264</v>
       </c>
       <c r="C508">
-        <v>384</v>
+        <v>634</v>
       </c>
       <c r="D508" t="s">
         <v>52</v>
       </c>
       <c r="E508">
-        <v>52.1</v>
+        <v>50.16</v>
       </c>
     </row>
     <row r="509" spans="1:5">
@@ -18090,16 +18090,16 @@
         <v>14</v>
       </c>
       <c r="B509">
-        <v>517</v>
+        <v>837</v>
       </c>
       <c r="C509">
-        <v>308</v>
+        <v>498</v>
       </c>
       <c r="D509" t="s">
         <v>53</v>
       </c>
       <c r="E509">
-        <v>59.57</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="510" spans="1:5">
@@ -18107,16 +18107,16 @@
         <v>14</v>
       </c>
       <c r="B510">
-        <v>233</v>
+        <v>393</v>
       </c>
       <c r="C510">
-        <v>123</v>
+        <v>217</v>
       </c>
       <c r="D510" t="s">
         <v>54</v>
       </c>
       <c r="E510">
-        <v>52.79</v>
+        <v>55.22</v>
       </c>
     </row>
     <row r="511" spans="1:5">
@@ -18124,16 +18124,16 @@
         <v>14</v>
       </c>
       <c r="B511">
-        <v>302</v>
+        <v>508</v>
       </c>
       <c r="C511">
-        <v>170</v>
+        <v>279</v>
       </c>
       <c r="D511" t="s">
         <v>55</v>
       </c>
       <c r="E511">
-        <v>56.29</v>
+        <v>54.92</v>
       </c>
     </row>
     <row r="512" spans="1:5">
@@ -18141,16 +18141,16 @@
         <v>14</v>
       </c>
       <c r="B512">
-        <v>379</v>
+        <v>618</v>
       </c>
       <c r="C512">
-        <v>224</v>
+        <v>350</v>
       </c>
       <c r="D512" t="s">
         <v>56</v>
       </c>
       <c r="E512">
-        <v>59.1</v>
+        <v>56.63</v>
       </c>
     </row>
     <row r="513" spans="1:5">
@@ -18158,16 +18158,16 @@
         <v>14</v>
       </c>
       <c r="B513">
-        <v>564</v>
+        <v>885</v>
       </c>
       <c r="C513">
-        <v>318</v>
+        <v>493</v>
       </c>
       <c r="D513" t="s">
         <v>57</v>
       </c>
       <c r="E513">
-        <v>56.38</v>
+        <v>55.71</v>
       </c>
     </row>
     <row r="514" spans="1:5">
@@ -18175,16 +18175,16 @@
         <v>14</v>
       </c>
       <c r="B514">
-        <v>172</v>
+        <v>256</v>
       </c>
       <c r="C514">
-        <v>99</v>
+        <v>146</v>
       </c>
       <c r="D514" t="s">
         <v>58</v>
       </c>
       <c r="E514">
-        <v>57.56</v>
+        <v>57.03</v>
       </c>
     </row>
     <row r="515" spans="1:5">
@@ -18192,16 +18192,16 @@
         <v>14</v>
       </c>
       <c r="B515">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="C515">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D515" t="s">
         <v>59</v>
       </c>
       <c r="E515">
-        <v>65.91</v>
+        <v>63.33</v>
       </c>
     </row>
     <row r="516" spans="1:5">
@@ -18209,16 +18209,16 @@
         <v>14</v>
       </c>
       <c r="B516">
-        <v>268</v>
+        <v>410</v>
       </c>
       <c r="C516">
-        <v>153</v>
+        <v>227</v>
       </c>
       <c r="D516" t="s">
         <v>60</v>
       </c>
       <c r="E516">
-        <v>57.09</v>
+        <v>55.37</v>
       </c>
     </row>
     <row r="517" spans="1:5">
@@ -18226,16 +18226,16 @@
         <v>14</v>
       </c>
       <c r="B517">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C517">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D517" t="s">
         <v>61</v>
       </c>
       <c r="E517">
-        <v>66.67</v>
+        <v>71.43000000000001</v>
       </c>
     </row>
     <row r="518" spans="1:5">
@@ -18243,16 +18243,16 @@
         <v>14</v>
       </c>
       <c r="B518">
-        <v>193</v>
+        <v>321</v>
       </c>
       <c r="C518">
-        <v>120</v>
+        <v>189</v>
       </c>
       <c r="D518" t="s">
         <v>62</v>
       </c>
       <c r="E518">
-        <v>62.18</v>
+        <v>58.88</v>
       </c>
     </row>
     <row r="519" spans="1:5">
@@ -18260,16 +18260,16 @@
         <v>14</v>
       </c>
       <c r="B519">
-        <v>797</v>
+        <v>1300</v>
       </c>
       <c r="C519">
-        <v>459</v>
+        <v>760</v>
       </c>
       <c r="D519" t="s">
         <v>63</v>
       </c>
       <c r="E519">
-        <v>57.59</v>
+        <v>58.46</v>
       </c>
     </row>
     <row r="520" spans="1:5">
@@ -18277,16 +18277,16 @@
         <v>14</v>
       </c>
       <c r="B520">
-        <v>118</v>
+        <v>206</v>
       </c>
       <c r="C520">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="D520" t="s">
         <v>64</v>
       </c>
       <c r="E520">
-        <v>55.08</v>
+        <v>52.43</v>
       </c>
     </row>
     <row r="521" spans="1:5">
@@ -18294,16 +18294,16 @@
         <v>14</v>
       </c>
       <c r="B521">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="C521">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="D521" t="s">
         <v>65</v>
       </c>
       <c r="E521">
-        <v>79.48999999999999</v>
+        <v>80.65000000000001</v>
       </c>
     </row>
     <row r="522" spans="1:5">
@@ -18311,16 +18311,16 @@
         <v>14</v>
       </c>
       <c r="B522">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C522">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D522" t="s">
         <v>66</v>
       </c>
       <c r="E522">
-        <v>33.33</v>
+        <v>31.25</v>
       </c>
     </row>
     <row r="523" spans="1:5">
@@ -18328,16 +18328,16 @@
         <v>14</v>
       </c>
       <c r="B523">
-        <v>212</v>
+        <v>345</v>
       </c>
       <c r="C523">
-        <v>128</v>
+        <v>206</v>
       </c>
       <c r="D523" t="s">
         <v>67</v>
       </c>
       <c r="E523">
-        <v>60.38</v>
+        <v>59.71</v>
       </c>
     </row>
   </sheetData>
@@ -18525,16 +18525,16 @@
         <v>14</v>
       </c>
       <c r="B11">
-        <v>12703</v>
+        <v>21009</v>
       </c>
       <c r="C11">
-        <v>6875</v>
+        <v>11577</v>
       </c>
       <c r="D11" t="s">
         <v>15</v>
       </c>
       <c r="E11">
-        <v>54.12</v>
+        <v>55.1</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -26362,16 +26362,16 @@
         <v>14</v>
       </c>
       <c r="B472">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="C472">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="D472" t="s">
         <v>16</v>
       </c>
       <c r="E472">
-        <v>44.44</v>
+        <v>65.12</v>
       </c>
     </row>
     <row r="473" spans="1:5">
@@ -26379,16 +26379,16 @@
         <v>14</v>
       </c>
       <c r="B473">
-        <v>210</v>
+        <v>350</v>
       </c>
       <c r="C473">
-        <v>120</v>
+        <v>202</v>
       </c>
       <c r="D473" t="s">
         <v>17</v>
       </c>
       <c r="E473">
-        <v>57.14</v>
+        <v>57.71</v>
       </c>
     </row>
     <row r="474" spans="1:5">
@@ -26396,16 +26396,16 @@
         <v>14</v>
       </c>
       <c r="B474">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="C474">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="D474" t="s">
         <v>18</v>
       </c>
       <c r="E474">
-        <v>53.85</v>
+        <v>48.61</v>
       </c>
     </row>
     <row r="475" spans="1:5">
@@ -26413,16 +26413,16 @@
         <v>14</v>
       </c>
       <c r="B475">
-        <v>183</v>
+        <v>305</v>
       </c>
       <c r="C475">
-        <v>105</v>
+        <v>176</v>
       </c>
       <c r="D475" t="s">
         <v>19</v>
       </c>
       <c r="E475">
-        <v>57.38</v>
+        <v>57.7</v>
       </c>
     </row>
     <row r="476" spans="1:5">
@@ -26430,16 +26430,16 @@
         <v>14</v>
       </c>
       <c r="B476">
-        <v>267</v>
+        <v>438</v>
       </c>
       <c r="C476">
-        <v>153</v>
+        <v>256</v>
       </c>
       <c r="D476" t="s">
         <v>20</v>
       </c>
       <c r="E476">
-        <v>57.3</v>
+        <v>58.45</v>
       </c>
     </row>
     <row r="477" spans="1:5">
@@ -26447,16 +26447,16 @@
         <v>14</v>
       </c>
       <c r="B477">
-        <v>355</v>
+        <v>602</v>
       </c>
       <c r="C477">
-        <v>181</v>
+        <v>312</v>
       </c>
       <c r="D477" t="s">
         <v>21</v>
       </c>
       <c r="E477">
-        <v>50.99</v>
+        <v>51.83</v>
       </c>
     </row>
     <row r="478" spans="1:5">
@@ -26464,16 +26464,16 @@
         <v>14</v>
       </c>
       <c r="B478">
-        <v>273</v>
+        <v>446</v>
       </c>
       <c r="C478">
-        <v>140</v>
+        <v>239</v>
       </c>
       <c r="D478" t="s">
         <v>22</v>
       </c>
       <c r="E478">
-        <v>51.28</v>
+        <v>53.59</v>
       </c>
     </row>
     <row r="479" spans="1:5">
@@ -26481,16 +26481,16 @@
         <v>14</v>
       </c>
       <c r="B479">
-        <v>97</v>
+        <v>141</v>
       </c>
       <c r="C479">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="D479" t="s">
         <v>23</v>
       </c>
       <c r="E479">
-        <v>41.24</v>
+        <v>36.17</v>
       </c>
     </row>
     <row r="480" spans="1:5">
@@ -26498,16 +26498,16 @@
         <v>14</v>
       </c>
       <c r="B480">
-        <v>292</v>
+        <v>492</v>
       </c>
       <c r="C480">
-        <v>141</v>
+        <v>247</v>
       </c>
       <c r="D480" t="s">
         <v>24</v>
       </c>
       <c r="E480">
-        <v>48.29</v>
+        <v>50.2</v>
       </c>
     </row>
     <row r="481" spans="1:5">
@@ -26515,16 +26515,16 @@
         <v>14</v>
       </c>
       <c r="B481">
-        <v>70</v>
+        <v>129</v>
       </c>
       <c r="C481">
-        <v>39</v>
+        <v>82</v>
       </c>
       <c r="D481" t="s">
         <v>25</v>
       </c>
       <c r="E481">
-        <v>55.71</v>
+        <v>63.57</v>
       </c>
     </row>
     <row r="482" spans="1:5">
@@ -26532,16 +26532,16 @@
         <v>14</v>
       </c>
       <c r="B482">
-        <v>345</v>
+        <v>568</v>
       </c>
       <c r="C482">
-        <v>211</v>
+        <v>347</v>
       </c>
       <c r="D482" t="s">
         <v>26</v>
       </c>
       <c r="E482">
-        <v>61.16</v>
+        <v>61.09</v>
       </c>
     </row>
     <row r="483" spans="1:5">
@@ -26549,16 +26549,16 @@
         <v>14</v>
       </c>
       <c r="B483">
-        <v>171</v>
+        <v>294</v>
       </c>
       <c r="C483">
-        <v>89</v>
+        <v>149</v>
       </c>
       <c r="D483" t="s">
         <v>27</v>
       </c>
       <c r="E483">
-        <v>52.05</v>
+        <v>50.68</v>
       </c>
     </row>
     <row r="484" spans="1:5">
@@ -26566,16 +26566,16 @@
         <v>14</v>
       </c>
       <c r="B484">
-        <v>286</v>
+        <v>480</v>
       </c>
       <c r="C484">
-        <v>175</v>
+        <v>297</v>
       </c>
       <c r="D484" t="s">
         <v>28</v>
       </c>
       <c r="E484">
-        <v>61.19</v>
+        <v>61.88</v>
       </c>
     </row>
     <row r="485" spans="1:5">
@@ -26583,16 +26583,16 @@
         <v>14</v>
       </c>
       <c r="B485">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="C485">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="D485" t="s">
         <v>29</v>
       </c>
       <c r="E485">
-        <v>45.88</v>
+        <v>44.22</v>
       </c>
     </row>
     <row r="486" spans="1:5">
@@ -26600,16 +26600,16 @@
         <v>14</v>
       </c>
       <c r="B486">
-        <v>186</v>
+        <v>296</v>
       </c>
       <c r="C486">
-        <v>87</v>
+        <v>141</v>
       </c>
       <c r="D486" t="s">
         <v>30</v>
       </c>
       <c r="E486">
-        <v>46.77</v>
+        <v>47.64</v>
       </c>
     </row>
     <row r="487" spans="1:5">
@@ -26617,16 +26617,16 @@
         <v>14</v>
       </c>
       <c r="B487">
-        <v>796</v>
+        <v>1317</v>
       </c>
       <c r="C487">
-        <v>454</v>
+        <v>753</v>
       </c>
       <c r="D487" t="s">
         <v>31</v>
       </c>
       <c r="E487">
-        <v>57.04</v>
+        <v>57.18</v>
       </c>
     </row>
     <row r="488" spans="1:5">
@@ -26634,16 +26634,16 @@
         <v>14</v>
       </c>
       <c r="B488">
-        <v>249</v>
+        <v>401</v>
       </c>
       <c r="C488">
-        <v>113</v>
+        <v>173</v>
       </c>
       <c r="D488" t="s">
         <v>32</v>
       </c>
       <c r="E488">
-        <v>45.38</v>
+        <v>43.14</v>
       </c>
     </row>
     <row r="489" spans="1:5">
@@ -26651,16 +26651,16 @@
         <v>14</v>
       </c>
       <c r="B489">
-        <v>273</v>
+        <v>505</v>
       </c>
       <c r="C489">
-        <v>128</v>
+        <v>238</v>
       </c>
       <c r="D489" t="s">
         <v>33</v>
       </c>
       <c r="E489">
-        <v>46.89</v>
+        <v>47.13</v>
       </c>
     </row>
     <row r="490" spans="1:5">
@@ -26668,16 +26668,16 @@
         <v>14</v>
       </c>
       <c r="B490">
-        <v>38</v>
+        <v>101</v>
       </c>
       <c r="C490">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="D490" t="s">
         <v>34</v>
       </c>
       <c r="E490">
-        <v>50</v>
+        <v>52.48</v>
       </c>
     </row>
     <row r="491" spans="1:5">
@@ -26685,16 +26685,16 @@
         <v>14</v>
       </c>
       <c r="B491">
-        <v>273</v>
+        <v>471</v>
       </c>
       <c r="C491">
-        <v>128</v>
+        <v>227</v>
       </c>
       <c r="D491" t="s">
         <v>35</v>
       </c>
       <c r="E491">
-        <v>46.89</v>
+        <v>48.2</v>
       </c>
     </row>
     <row r="492" spans="1:5">
@@ -26702,16 +26702,16 @@
         <v>14</v>
       </c>
       <c r="B492">
-        <v>72</v>
+        <v>113</v>
       </c>
       <c r="C492">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="D492" t="s">
         <v>36</v>
       </c>
       <c r="E492">
-        <v>56.94</v>
+        <v>53.1</v>
       </c>
     </row>
     <row r="493" spans="1:5">
@@ -26719,16 +26719,16 @@
         <v>14</v>
       </c>
       <c r="B493">
-        <v>94</v>
+        <v>146</v>
       </c>
       <c r="C493">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="D493" t="s">
         <v>37</v>
       </c>
       <c r="E493">
-        <v>48.94</v>
+        <v>45.21</v>
       </c>
     </row>
     <row r="494" spans="1:5">
@@ -26736,16 +26736,16 @@
         <v>14</v>
       </c>
       <c r="B494">
-        <v>193</v>
+        <v>332</v>
       </c>
       <c r="C494">
-        <v>105</v>
+        <v>196</v>
       </c>
       <c r="D494" t="s">
         <v>38</v>
       </c>
       <c r="E494">
-        <v>54.4</v>
+        <v>59.04</v>
       </c>
     </row>
     <row r="495" spans="1:5">
@@ -26753,16 +26753,16 @@
         <v>14</v>
       </c>
       <c r="B495">
-        <v>227</v>
+        <v>338</v>
       </c>
       <c r="C495">
-        <v>144</v>
+        <v>215</v>
       </c>
       <c r="D495" t="s">
         <v>39</v>
       </c>
       <c r="E495">
-        <v>63.44</v>
+        <v>63.61</v>
       </c>
     </row>
     <row r="496" spans="1:5">
@@ -26770,16 +26770,16 @@
         <v>14</v>
       </c>
       <c r="B496">
-        <v>143</v>
+        <v>230</v>
       </c>
       <c r="C496">
-        <v>80</v>
+        <v>128</v>
       </c>
       <c r="D496" t="s">
         <v>40</v>
       </c>
       <c r="E496">
-        <v>55.94</v>
+        <v>55.65</v>
       </c>
     </row>
     <row r="497" spans="1:5">
@@ -26787,16 +26787,16 @@
         <v>14</v>
       </c>
       <c r="B497">
-        <v>744</v>
+        <v>1216</v>
       </c>
       <c r="C497">
-        <v>381</v>
+        <v>625</v>
       </c>
       <c r="D497" t="s">
         <v>41</v>
       </c>
       <c r="E497">
-        <v>51.21</v>
+        <v>51.4</v>
       </c>
     </row>
     <row r="498" spans="1:5">
@@ -26804,16 +26804,16 @@
         <v>14</v>
       </c>
       <c r="B498">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="C498">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="D498" t="s">
         <v>42</v>
       </c>
       <c r="E498">
-        <v>40</v>
+        <v>48.28</v>
       </c>
     </row>
     <row r="499" spans="1:5">
@@ -26821,16 +26821,16 @@
         <v>14</v>
       </c>
       <c r="B499">
-        <v>352</v>
+        <v>542</v>
       </c>
       <c r="C499">
-        <v>223</v>
+        <v>351</v>
       </c>
       <c r="D499" t="s">
         <v>43</v>
       </c>
       <c r="E499">
-        <v>63.35</v>
+        <v>64.76000000000001</v>
       </c>
     </row>
     <row r="500" spans="1:5">
@@ -26838,16 +26838,16 @@
         <v>14</v>
       </c>
       <c r="B500">
-        <v>161</v>
+        <v>254</v>
       </c>
       <c r="C500">
-        <v>99</v>
+        <v>156</v>
       </c>
       <c r="D500" t="s">
         <v>44</v>
       </c>
       <c r="E500">
-        <v>61.49</v>
+        <v>61.42</v>
       </c>
     </row>
     <row r="501" spans="1:5">
@@ -26855,16 +26855,16 @@
         <v>14</v>
       </c>
       <c r="B501">
-        <v>216</v>
+        <v>318</v>
       </c>
       <c r="C501">
-        <v>124</v>
+        <v>177</v>
       </c>
       <c r="D501" t="s">
         <v>45</v>
       </c>
       <c r="E501">
-        <v>57.41</v>
+        <v>55.66</v>
       </c>
     </row>
     <row r="502" spans="1:5">
@@ -26872,16 +26872,16 @@
         <v>14</v>
       </c>
       <c r="B502">
-        <v>210</v>
+        <v>335</v>
       </c>
       <c r="C502">
-        <v>110</v>
+        <v>179</v>
       </c>
       <c r="D502" t="s">
         <v>46</v>
       </c>
       <c r="E502">
-        <v>52.38</v>
+        <v>53.43</v>
       </c>
     </row>
     <row r="503" spans="1:5">
@@ -26889,16 +26889,16 @@
         <v>14</v>
       </c>
       <c r="B503">
-        <v>179</v>
+        <v>280</v>
       </c>
       <c r="C503">
-        <v>104</v>
+        <v>164</v>
       </c>
       <c r="D503" t="s">
         <v>47</v>
       </c>
       <c r="E503">
-        <v>58.1</v>
+        <v>58.57</v>
       </c>
     </row>
     <row r="504" spans="1:5">
@@ -26906,16 +26906,16 @@
         <v>14</v>
       </c>
       <c r="B504">
-        <v>390</v>
+        <v>648</v>
       </c>
       <c r="C504">
-        <v>227</v>
+        <v>376</v>
       </c>
       <c r="D504" t="s">
         <v>48</v>
       </c>
       <c r="E504">
-        <v>58.21</v>
+        <v>58.02</v>
       </c>
     </row>
     <row r="505" spans="1:5">
@@ -26923,16 +26923,16 @@
         <v>14</v>
       </c>
       <c r="B505">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="C505">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="D505" t="s">
         <v>49</v>
       </c>
       <c r="E505">
-        <v>65.62</v>
+        <v>59.65</v>
       </c>
     </row>
     <row r="506" spans="1:5">
@@ -26940,16 +26940,16 @@
         <v>14</v>
       </c>
       <c r="B506">
-        <v>54</v>
+        <v>80</v>
       </c>
       <c r="C506">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="D506" t="s">
         <v>50</v>
       </c>
       <c r="E506">
-        <v>72.22</v>
+        <v>75</v>
       </c>
     </row>
     <row r="507" spans="1:5">
@@ -26957,16 +26957,16 @@
         <v>14</v>
       </c>
       <c r="B507">
-        <v>402</v>
+        <v>650</v>
       </c>
       <c r="C507">
-        <v>254</v>
+        <v>408</v>
       </c>
       <c r="D507" t="s">
         <v>51</v>
       </c>
       <c r="E507">
-        <v>63.18</v>
+        <v>62.77</v>
       </c>
     </row>
     <row r="508" spans="1:5">
@@ -26974,16 +26974,16 @@
         <v>14</v>
       </c>
       <c r="B508">
-        <v>811</v>
+        <v>1387</v>
       </c>
       <c r="C508">
-        <v>367</v>
+        <v>637</v>
       </c>
       <c r="D508" t="s">
         <v>52</v>
       </c>
       <c r="E508">
-        <v>45.25</v>
+        <v>45.93</v>
       </c>
     </row>
     <row r="509" spans="1:5">
@@ -26991,16 +26991,16 @@
         <v>14</v>
       </c>
       <c r="B509">
-        <v>393</v>
+        <v>704</v>
       </c>
       <c r="C509">
-        <v>207</v>
+        <v>385</v>
       </c>
       <c r="D509" t="s">
         <v>53</v>
       </c>
       <c r="E509">
-        <v>52.67</v>
+        <v>54.69</v>
       </c>
     </row>
     <row r="510" spans="1:5">
@@ -27008,16 +27008,16 @@
         <v>14</v>
       </c>
       <c r="B510">
-        <v>347</v>
+        <v>500</v>
       </c>
       <c r="C510">
-        <v>196</v>
+        <v>271</v>
       </c>
       <c r="D510" t="s">
         <v>54</v>
       </c>
       <c r="E510">
-        <v>56.48</v>
+        <v>54.2</v>
       </c>
     </row>
     <row r="511" spans="1:5">
@@ -27025,16 +27025,16 @@
         <v>14</v>
       </c>
       <c r="B511">
-        <v>323</v>
+        <v>520</v>
       </c>
       <c r="C511">
-        <v>154</v>
+        <v>259</v>
       </c>
       <c r="D511" t="s">
         <v>55</v>
       </c>
       <c r="E511">
-        <v>47.68</v>
+        <v>49.81</v>
       </c>
     </row>
     <row r="512" spans="1:5">
@@ -27042,16 +27042,16 @@
         <v>14</v>
       </c>
       <c r="B512">
-        <v>313</v>
+        <v>530</v>
       </c>
       <c r="C512">
-        <v>203</v>
+        <v>349</v>
       </c>
       <c r="D512" t="s">
         <v>56</v>
       </c>
       <c r="E512">
-        <v>64.86</v>
+        <v>65.84999999999999</v>
       </c>
     </row>
     <row r="513" spans="1:5">
@@ -27059,16 +27059,16 @@
         <v>14</v>
       </c>
       <c r="B513">
-        <v>697</v>
+        <v>1159</v>
       </c>
       <c r="C513">
-        <v>363</v>
+        <v>657</v>
       </c>
       <c r="D513" t="s">
         <v>57</v>
       </c>
       <c r="E513">
-        <v>52.08</v>
+        <v>56.69</v>
       </c>
     </row>
     <row r="514" spans="1:5">
@@ -27076,16 +27076,16 @@
         <v>14</v>
       </c>
       <c r="B514">
-        <v>180</v>
+        <v>298</v>
       </c>
       <c r="C514">
-        <v>75</v>
+        <v>136</v>
       </c>
       <c r="D514" t="s">
         <v>58</v>
       </c>
       <c r="E514">
-        <v>41.67</v>
+        <v>45.64</v>
       </c>
     </row>
     <row r="515" spans="1:5">
@@ -27093,16 +27093,16 @@
         <v>14</v>
       </c>
       <c r="B515">
-        <v>34</v>
+        <v>64</v>
       </c>
       <c r="C515">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="D515" t="s">
         <v>59</v>
       </c>
       <c r="E515">
-        <v>58.82</v>
+        <v>56.25</v>
       </c>
     </row>
     <row r="516" spans="1:5">
@@ -27110,16 +27110,16 @@
         <v>14</v>
       </c>
       <c r="B516">
-        <v>268</v>
+        <v>446</v>
       </c>
       <c r="C516">
-        <v>159</v>
+        <v>258</v>
       </c>
       <c r="D516" t="s">
         <v>60</v>
       </c>
       <c r="E516">
-        <v>59.33</v>
+        <v>57.85</v>
       </c>
     </row>
     <row r="517" spans="1:5">
@@ -27127,16 +27127,16 @@
         <v>14</v>
       </c>
       <c r="B517">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="C517">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="D517" t="s">
         <v>61</v>
       </c>
       <c r="E517">
-        <v>37.74</v>
+        <v>56.96</v>
       </c>
     </row>
     <row r="518" spans="1:5">
@@ -27144,16 +27144,16 @@
         <v>14</v>
       </c>
       <c r="B518">
-        <v>181</v>
+        <v>279</v>
       </c>
       <c r="C518">
-        <v>95</v>
+        <v>171</v>
       </c>
       <c r="D518" t="s">
         <v>62</v>
       </c>
       <c r="E518">
-        <v>52.49</v>
+        <v>61.29</v>
       </c>
     </row>
     <row r="519" spans="1:5">
@@ -27161,16 +27161,16 @@
         <v>14</v>
       </c>
       <c r="B519">
-        <v>744</v>
+        <v>1282</v>
       </c>
       <c r="C519">
-        <v>428</v>
+        <v>736</v>
       </c>
       <c r="D519" t="s">
         <v>63</v>
       </c>
       <c r="E519">
-        <v>57.53</v>
+        <v>57.41</v>
       </c>
     </row>
     <row r="520" spans="1:5">
@@ -27178,16 +27178,16 @@
         <v>14</v>
       </c>
       <c r="B520">
-        <v>92</v>
+        <v>155</v>
       </c>
       <c r="C520">
-        <v>42</v>
+        <v>96</v>
       </c>
       <c r="D520" t="s">
         <v>64</v>
       </c>
       <c r="E520">
-        <v>45.65</v>
+        <v>61.94</v>
       </c>
     </row>
     <row r="521" spans="1:5">
@@ -27195,16 +27195,16 @@
         <v>14</v>
       </c>
       <c r="B521">
-        <v>36</v>
+        <v>72</v>
       </c>
       <c r="C521">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="D521" t="s">
         <v>65</v>
       </c>
       <c r="E521">
-        <v>58.33</v>
+        <v>61.11</v>
       </c>
     </row>
     <row r="522" spans="1:5">
@@ -27212,16 +27212,16 @@
         <v>14</v>
       </c>
       <c r="B522">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C522">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D522" t="s">
         <v>66</v>
       </c>
       <c r="E522">
-        <v>36.84</v>
+        <v>39.29</v>
       </c>
     </row>
     <row r="523" spans="1:5">
@@ -27229,16 +27229,16 @@
         <v>14</v>
       </c>
       <c r="B523">
-        <v>202</v>
+        <v>311</v>
       </c>
       <c r="C523">
-        <v>115</v>
+        <v>192</v>
       </c>
       <c r="D523" t="s">
         <v>67</v>
       </c>
       <c r="E523">
-        <v>56.93</v>
+        <v>61.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>